<commit_message>
Add group-based changeover setup times
</commit_message>
<xml_diff>
--- a/data/EastFu_Lean_APS_Demo.xlsx
+++ b/data/EastFu_Lean_APS_Demo.xlsx
@@ -11,6 +11,8 @@
     <sheet name="產品機台產速" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="機台可用時間" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="排程基本設定" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="機台初始狀態" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="換模時間" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -432,8 +434,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -466,6 +477,11 @@
           <t>交期</t>
         </is>
       </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>允許機台</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -496,6 +512,7 @@
           <t>2026-09-04</t>
         </is>
       </c>
+      <c r="G2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -526,6 +543,7 @@
           <t>2026-09-04</t>
         </is>
       </c>
+      <c r="G3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -556,6 +574,7 @@
           <t>2026-09-04</t>
         </is>
       </c>
+      <c r="G4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -586,6 +605,7 @@
           <t>2026-09-04</t>
         </is>
       </c>
+      <c r="G5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -616,6 +636,7 @@
           <t>2026-09-05</t>
         </is>
       </c>
+      <c r="G6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -646,6 +667,7 @@
           <t>2026-09-05</t>
         </is>
       </c>
+      <c r="G7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -676,6 +698,7 @@
           <t>2026-09-04</t>
         </is>
       </c>
+      <c r="G8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -706,6 +729,7 @@
           <t>2026-09-05</t>
         </is>
       </c>
+      <c r="G9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -736,6 +760,11 @@
           <t>2026-09-04</t>
         </is>
       </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>C2,C5</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -766,6 +795,7 @@
           <t>2026-09-05</t>
         </is>
       </c>
+      <c r="G11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -778,8 +808,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -797,6 +833,11 @@
           <t>產速_PCS_per_hr</t>
         </is>
       </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>換模群組</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -812,6 +853,11 @@
       <c r="C2" t="n">
         <v>120</v>
       </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>C2-A</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -827,6 +873,11 @@
       <c r="C3" t="n">
         <v>96</v>
       </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>C2-B</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -842,6 +893,11 @@
       <c r="C4" t="n">
         <v>90</v>
       </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>MULTI-A</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -857,6 +913,11 @@
       <c r="C5" t="n">
         <v>84</v>
       </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>MULTI-A</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -872,6 +933,11 @@
       <c r="C6" t="n">
         <v>144</v>
       </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>C4-A</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -887,6 +953,11 @@
       <c r="C7" t="n">
         <v>108</v>
       </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>C4-B</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -902,6 +973,11 @@
       <c r="C8" t="n">
         <v>84</v>
       </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>MULTI-B</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -917,6 +993,11 @@
       <c r="C9" t="n">
         <v>78</v>
       </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>MULTI-B</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -932,6 +1013,11 @@
       <c r="C10" t="n">
         <v>150</v>
       </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>C5-A</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -947,6 +1033,11 @@
       <c r="C11" t="n">
         <v>110</v>
       </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>C5-B</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -962,6 +1053,11 @@
       <c r="C12" t="n">
         <v>100</v>
       </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>MULTI-C</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -977,6 +1073,11 @@
       <c r="C13" t="n">
         <v>92</v>
       </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>MULTI-C</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -991,6 +1092,11 @@
       </c>
       <c r="C14" t="n">
         <v>140</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>C2-C</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -1006,6 +1112,11 @@
   </sheetPr>
   <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="3" max="3"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -1076,6 +1187,10 @@
   </sheetPr>
   <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -1131,6 +1246,273 @@
         <is>
           <t>是</t>
         </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>機台</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>初始產品</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>SIM-C2-A</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>SIM-C4-A</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>C5</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>SIM-C5-A</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>來源換模群組</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>目標換模群組</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>換模時間_分鐘</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>C2-A</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>C2-B</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>C2-B</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>C2-A</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>C2-A</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>C2-C</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>C2-C</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>C2-A</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>C4-A</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>C4-B</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>C4-B</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>C4-A</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>C5-A</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>C5-B</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>C5-B</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>C5-A</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>MULTI-A</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>MULTI-B</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>MULTI-B</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>MULTI-C</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>MULTI-C</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>MULTI-A</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Move schedule settings into the app
</commit_message>
<xml_diff>
--- a/data/EastFu_Lean_APS_Demo.xlsx
+++ b/data/EastFu_Lean_APS_Demo.xlsx
@@ -10,9 +10,8 @@
     <sheet name="待排工單" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="產品機台產速" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="機台可用時間" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="排程基本設定" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="機台初始狀態" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="換模時間" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="機台初始狀態" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="換模時間" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1185,80 +1184,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="21" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>設定項目</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>設定值</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>排程開始</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="n">
-        <v>46268.33333333334</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>排程結束</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="n">
-        <v>46269.33333333334</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>時區</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Asia/Taipei</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>允許跨班</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1319,7 +1244,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Simplify availability setup in the app
</commit_message>
<xml_diff>
--- a/data/EastFu_Lean_APS_Demo.xlsx
+++ b/data/EastFu_Lean_APS_Demo.xlsx
@@ -9,9 +9,8 @@
   <sheets>
     <sheet name="待排工單" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="產品機台產速" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="機台可用時間" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="機台初始狀態" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="換模時間" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="機台初始狀態" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="換模時間" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,10 +19,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="2">
     <font>
       <name val="Calibri"/>
@@ -62,12 +58,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1109,81 +1104,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="21" customWidth="1" min="2" max="2"/>
-    <col width="21" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>機台</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>可用開始</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>可用結束</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>C2</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="n">
-        <v>46268.33333333334</v>
-      </c>
-      <c r="C2" s="2" t="n">
-        <v>46269.33333333334</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>C4</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="n">
-        <v>46268.33333333334</v>
-      </c>
-      <c r="C3" s="2" t="n">
-        <v>46269.33333333334</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>C5</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="n">
-        <v>46268.33333333334</v>
-      </c>
-      <c r="C4" s="2" t="n">
-        <v>46269.33333333334</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1244,7 +1164,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Add machine and workforce scheduling controls
</commit_message>
<xml_diff>
--- a/data/EastFu_Lean_APS_Demo.xlsx
+++ b/data/EastFu_Lean_APS_Demo.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="待排工單" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="產品機台產速" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="機台初始狀態" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="換模時間" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="待排工單" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="產品機台產速" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="機台初始狀態" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="換模時間" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -29,18 +29,33 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <family val="2"/>
       <b val="1"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4EC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E5E7EB"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -48,21 +63,14 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -471,9 +479,9 @@
           <t>交期</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>允許機台</t>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>工單限定機台</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add workbook guide and assistant manual
</commit_message>
<xml_diff>
--- a/data/EastFu_Lean_APS_Demo.xlsx
+++ b/data/EastFu_Lean_APS_Demo.xlsx
@@ -11,6 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="產品機台產速" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="機台初始狀態" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="換模時間" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填表說明" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -37,7 +38,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -46,12 +47,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FCE4EC"/>
+        <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00E5E7EB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -67,10 +73,25 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1371,4 +1392,514 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="58" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="48" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>工作表</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>欄位</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>必填</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>定義</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>範例</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>備註</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>待排工單</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>工單編號</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>工單或製令的唯一編號。系統用它識別每一張工單，不可重複。</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>WO-20260905-001</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>待排工單</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>產品</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>要生產的產品代號，必須能在產品機台產速表找到對應產速。</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>SIM-C2-A</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>待排工單</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>數量</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>本工單要生產的數量。必須大於 0。</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>600</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>待排工單</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>單位</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>數量單位。目前排程時間以 PCS/hr 產速換算。</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>PCS</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>待排工單</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>優先級</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>工單急迫程度。支援急單、一般、低優先。</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>急單</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>待排工單</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>交期</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>工單需要完成的時間。只填日期時，系統視為當天 23:59:59。</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>2026/09/05 18:00</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>若只填 2026/09/05，代表 2026/09/05 23:59:59。</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>待排工單</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>工單限定機台</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>單張工單的特殊限制。空白代表依產品機台產速表判斷；若填 C2,C5，代表這張工單只能排在 C2 或 C5。</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>C2,C5</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>產品機台產速</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>產品</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>產品代號。每個可生產的產品/機台組合各填一列。</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>SIM-C2-A</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>產品機台產速</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>機台</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>可生產該產品的機台。</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>產品機台產速</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>產速_PCS_per_hr</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>標準產速，每小時可生產 PCS 數。系統用數量除以產速計算加工時間。</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>120</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>產品機台產速</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>換模群組</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>產品族群或模具/換線分類。前後工單群組不同時，系統會計算換模時間。</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>C2-A</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>機台初始狀態</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>機台</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>排程開始前的機台。用來判斷第一張工單是否需要換模。</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>機台初始狀態</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>初始產品</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>排程開始前，該機台正在做或最後做的產品。</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>SIM-C2-A</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>若不確定，可留空或填目前最接近的產品。</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>換模時間</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>來源換模群組</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>上一張工單的換模群組。</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>C2-A</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>換模時間</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>目標換模群組</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>下一張工單的換模群組。</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>C2-B</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>換模時間</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>換模時間_分鐘</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>從來源群組切換到目標群組需要的分鐘數。</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Make machine initial state optional
</commit_message>
<xml_diff>
--- a/data/EastFu_Lean_APS_Demo.xlsx
+++ b/data/EastFu_Lean_APS_Demo.xlsx
@@ -1133,7 +1133,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1141,50 +1141,14 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>機台</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>初始產品</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>C2</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>SIM-C2-A</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>C4</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>SIM-C4-A</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>C5</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>SIM-C5-A</t>
         </is>
       </c>
     </row>
@@ -1633,7 +1597,7 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>單張工單的特殊限制。空白代表依產品機台產速表判斷；若填 C2,C5，代表這張工單只能排在 C2 或 C5。</t>
+          <t>單張工單的特殊限制。空白代表依產品機台產速表判斷；若填 C2,C5，代表這張工單只能排在 C2 或 C5。欄名也可用限定機台、允許機台、可排機台。</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -1766,14 +1730,14 @@
           <t>機台</t>
         </is>
       </c>
-      <c r="C13" s="6" t="inlineStr">
-        <is>
-          <t>是</t>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>否</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>排程開始前的機台。用來判斷第一張工單是否需要換模。</t>
+          <t>進階選填。若要告訴系統排程開始前某台機台最後做的是什麼產品，才需要填。</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
@@ -1794,14 +1758,14 @@
           <t>初始產品</t>
         </is>
       </c>
-      <c r="C14" s="6" t="inlineStr">
-        <is>
-          <t>是</t>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>否</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>排程開始前，該機台正在做或最後做的產品。</t>
+          <t>進階選填。若空白，系統視為空機台，第一張工單不計換模。</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
@@ -1811,7 +1775,7 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>若不確定，可留空或填目前最接近的產品。</t>
+          <t>一般從新訂單重新排程時可整張表留空；不是用來指定某張工單一定要排在哪台。</t>
         </is>
       </c>
     </row>

</xml_diff>